<commit_message>
Added new folder practice for excel
</commit_message>
<xml_diff>
--- a/Excel/V-Lookup.xlsx
+++ b/Excel/V-Lookup.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Abror All Materials\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Arbor all Folder\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47EBAA37-D3CD-4F66-9642-817FD385573C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6A7B95-520B-4B59-818F-F98EB66AA363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{87CFD858-0C59-4A7A-89DF-5A43856E8BAC}"/>
   </bookViews>
@@ -2160,11 +2160,11 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B37" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C37" s="1" t="str">
         <f>VLOOKUP(B37,$A$1:$L$31,4)</f>
-        <v>Printer</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>